<commit_message>
added abelization for 40 lines
</commit_message>
<xml_diff>
--- a/results/5105_bef_gauss.xlsx
+++ b/results/5105_bef_gauss.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T11"/>
+  <dimension ref="A1:T15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -435,681 +435,929 @@
         </is>
       </c>
       <c r="B1" s="1" t="n">
-        <v>-3.3015</v>
+        <v>-2.976</v>
       </c>
       <c r="C1" s="1" t="n">
-        <v>-2.945</v>
+        <v>-2.6505</v>
       </c>
       <c r="D1" s="1" t="n">
-        <v>-2.573</v>
+        <v>-2.325</v>
       </c>
       <c r="E1" s="1" t="n">
-        <v>-2.201</v>
+        <v>-1.984</v>
       </c>
       <c r="F1" s="1" t="n">
-        <v>-1.8445</v>
+        <v>-1.6585</v>
       </c>
       <c r="G1" s="1" t="n">
-        <v>-1.4725</v>
+        <v>-1.333</v>
       </c>
       <c r="H1" s="1" t="n">
-        <v>-1.1005</v>
+        <v>-0.992</v>
       </c>
       <c r="I1" s="1" t="n">
-        <v>-0.744</v>
+        <v>-0.6665</v>
       </c>
       <c r="J1" s="1" t="n">
-        <v>-0.372</v>
+        <v>-0.341</v>
       </c>
       <c r="K1" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L1" s="1" t="n">
-        <v>0.31</v>
+        <v>0.2635</v>
       </c>
       <c r="M1" s="1" t="n">
-        <v>0.62</v>
+        <v>0.527</v>
       </c>
       <c r="N1" s="1" t="n">
-        <v>0.9455</v>
+        <v>0.7905</v>
       </c>
       <c r="O1" s="1" t="n">
-        <v>1.2555</v>
+        <v>1.054</v>
       </c>
       <c r="P1" s="1" t="n">
-        <v>1.5655</v>
+        <v>1.3175</v>
       </c>
       <c r="Q1" s="1" t="n">
-        <v>1.891</v>
+        <v>1.581</v>
       </c>
       <c r="R1" s="1" t="n">
-        <v>2.201</v>
+        <v>1.8445</v>
       </c>
       <c r="S1" s="1" t="n">
-        <v>2.511</v>
+        <v>2.108</v>
       </c>
       <c r="T1" s="1" t="n">
-        <v>2.8365</v>
+        <v>2.387</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>509.97454</v>
+        <v>509.5793</v>
       </c>
       <c r="B2" t="n">
-        <v>0.06282039067999266</v>
+        <v>0.05510467262052601</v>
       </c>
       <c r="C2" t="n">
-        <v>-0.1083793365031144</v>
+        <v>0.04753978951075966</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.1733776400475411</v>
+        <v>0.09107001945560603</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.7099883252063507</v>
+        <v>0.1096854205230304</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.09543888715996908</v>
+        <v>0.09536850919764456</v>
       </c>
       <c r="G2" t="n">
-        <v>1.781960929869342</v>
+        <v>0.146991553986824</v>
       </c>
       <c r="H2" t="n">
-        <v>3.735194320606352</v>
+        <v>0.1674117186763795</v>
       </c>
       <c r="I2" t="n">
-        <v>5.560491209038316</v>
+        <v>0.1557483543283996</v>
       </c>
       <c r="J2" t="n">
-        <v>8.12523971143203</v>
+        <v>0.1651802864685875</v>
       </c>
       <c r="K2" t="n">
-        <v>9.486181196016144</v>
+        <v>0.159150164106019</v>
       </c>
       <c r="L2" t="n">
-        <v>8.750097868742191</v>
+        <v>0.1570590719515982</v>
       </c>
       <c r="M2" t="n">
-        <v>6.811282138237561</v>
+        <v>0.1650194848034033</v>
       </c>
       <c r="N2" t="n">
-        <v>4.725046497728611</v>
+        <v>0.1687432387760058</v>
       </c>
       <c r="O2" t="n">
-        <v>2.79482051292872</v>
+        <v>0.1442294920334351</v>
       </c>
       <c r="P2" t="n">
-        <v>0.6466014313212646</v>
+        <v>0.1160845450417988</v>
       </c>
       <c r="Q2" t="n">
-        <v>-0.6244012668409518</v>
+        <v>0.09955178491370892</v>
       </c>
       <c r="R2" t="n">
-        <v>-0.6735938236378025</v>
+        <v>0.09056285100871049</v>
       </c>
       <c r="S2" t="n">
-        <v>-0.1517542229532488</v>
+        <v>0.07227985309375015</v>
       </c>
       <c r="T2" t="n">
-        <v>0.3300480454261971</v>
+        <v>0.05079114875644523</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>510.06962</v>
+        <v>509.676</v>
       </c>
       <c r="B3" t="n">
-        <v>0.1147525537666079</v>
+        <v>0.03549753212595357</v>
       </c>
       <c r="C3" t="n">
-        <v>0.7819688276866791</v>
+        <v>0.05813147694004187</v>
       </c>
       <c r="D3" t="n">
-        <v>3.220027508768816</v>
+        <v>0.06477230988079928</v>
       </c>
       <c r="E3" t="n">
-        <v>5.90880843845934</v>
+        <v>0.07330058693470362</v>
       </c>
       <c r="F3" t="n">
-        <v>7.975145838485807</v>
+        <v>0.09589603055683323</v>
       </c>
       <c r="G3" t="n">
-        <v>10.98933339432313</v>
+        <v>0.1242319282049364</v>
       </c>
       <c r="H3" t="n">
-        <v>14.41017684833845</v>
+        <v>0.1203421487635561</v>
       </c>
       <c r="I3" t="n">
-        <v>16.37691972063788</v>
+        <v>0.126499431474817</v>
       </c>
       <c r="J3" t="n">
-        <v>17.25424742905898</v>
+        <v>0.1440641140010566</v>
       </c>
       <c r="K3" t="n">
-        <v>16.62650038200992</v>
+        <v>0.1659228901689966</v>
       </c>
       <c r="L3" t="n">
-        <v>16.03322619796337</v>
+        <v>0.183262200199239</v>
       </c>
       <c r="M3" t="n">
-        <v>14.93759117537581</v>
+        <v>0.1652033900017666</v>
       </c>
       <c r="N3" t="n">
-        <v>13.13548770714882</v>
+        <v>0.1347509410709737</v>
       </c>
       <c r="O3" t="n">
-        <v>11.17251053696176</v>
+        <v>0.1182452363493951</v>
       </c>
       <c r="P3" t="n">
-        <v>8.742006808540614</v>
+        <v>0.0957968926383134</v>
       </c>
       <c r="Q3" t="n">
-        <v>6.297688338792088</v>
+        <v>0.07129641164916739</v>
       </c>
       <c r="R3" t="n">
-        <v>4.13982123853697</v>
+        <v>0.03790942757516173</v>
       </c>
       <c r="S3" t="n">
-        <v>2.037262248154017</v>
+        <v>0.03325763174523857</v>
       </c>
       <c r="T3" t="n">
-        <v>0.4575143774410473</v>
+        <v>0.0357887016758557</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>510.16469</v>
+        <v>509.7727</v>
       </c>
       <c r="B4" t="n">
-        <v>1.688284545800363</v>
+        <v>0.04330342277174554</v>
       </c>
       <c r="C4" t="n">
-        <v>1.691028834464588</v>
+        <v>0.06163012557907382</v>
       </c>
       <c r="D4" t="n">
-        <v>-1.346676842527556</v>
+        <v>0.08349809744884623</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.6603091848821658</v>
+        <v>0.09117528758583196</v>
       </c>
       <c r="F4" t="n">
-        <v>4.296966087464287</v>
+        <v>0.09964577346378899</v>
       </c>
       <c r="G4" t="n">
-        <v>9.083430862169749</v>
+        <v>0.1194248403202188</v>
       </c>
       <c r="H4" t="n">
-        <v>14.36329706250363</v>
+        <v>0.1368144013164815</v>
       </c>
       <c r="I4" t="n">
-        <v>18.6538103907429</v>
+        <v>0.1726521469204638</v>
       </c>
       <c r="J4" t="n">
-        <v>21.32647250735615</v>
+        <v>0.1769600911937245</v>
       </c>
       <c r="K4" t="n">
-        <v>20.87227023925722</v>
+        <v>0.1724412220601187</v>
       </c>
       <c r="L4" t="n">
-        <v>18.01508640630429</v>
+        <v>0.154032096580668</v>
       </c>
       <c r="M4" t="n">
-        <v>14.47482724413324</v>
+        <v>0.1312351832271739</v>
       </c>
       <c r="N4" t="n">
-        <v>11.00682446631847</v>
+        <v>0.1245856908663845</v>
       </c>
       <c r="O4" t="n">
-        <v>6.927281907759498</v>
+        <v>0.1323486637395381</v>
       </c>
       <c r="P4" t="n">
-        <v>1.859890519067573</v>
+        <v>0.1308491447002214</v>
       </c>
       <c r="Q4" t="n">
-        <v>-2.577080301073288</v>
+        <v>0.1051989701832335</v>
       </c>
       <c r="R4" t="n">
-        <v>-3.313786842401943</v>
+        <v>0.09461449728517345</v>
       </c>
       <c r="S4" t="n">
-        <v>-1.741267516847894</v>
+        <v>0.07395417332858364</v>
       </c>
       <c r="T4" t="n">
-        <v>0.09973505717710447</v>
+        <v>0.04542423963707185</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>510.25975</v>
+        <v>509.8694</v>
       </c>
       <c r="B5" t="n">
-        <v>-1.439878207539081</v>
+        <v>0.04124633755559197</v>
       </c>
       <c r="C5" t="n">
-        <v>1.537877384988718</v>
+        <v>0.0527996393595406</v>
       </c>
       <c r="D5" t="n">
-        <v>15.71016571117021</v>
+        <v>0.07623661011919013</v>
       </c>
       <c r="E5" t="n">
-        <v>40.98771617015807</v>
+        <v>0.08695303548834073</v>
       </c>
       <c r="F5" t="n">
-        <v>75.33769238164857</v>
+        <v>0.09192812570716265</v>
       </c>
       <c r="G5" t="n">
-        <v>128.6711669247999</v>
+        <v>0.1091717898309827</v>
       </c>
       <c r="H5" t="n">
-        <v>194.5086975652391</v>
+        <v>0.1390342764063229</v>
       </c>
       <c r="I5" t="n">
-        <v>255.0664195266429</v>
+        <v>0.1305202837217479</v>
       </c>
       <c r="J5" t="n">
-        <v>313.6909062429291</v>
+        <v>0.1181549752357143</v>
       </c>
       <c r="K5" t="n">
-        <v>346.9530990380694</v>
+        <v>0.1294298690126215</v>
       </c>
       <c r="L5" t="n">
-        <v>336.3877528177557</v>
+        <v>0.1219503287386494</v>
       </c>
       <c r="M5" t="n">
-        <v>296.7783982486488</v>
+        <v>0.1210326196762051</v>
       </c>
       <c r="N5" t="n">
-        <v>228.9153508168242</v>
+        <v>0.1298467982849929</v>
       </c>
       <c r="O5" t="n">
-        <v>154.5526768915494</v>
+        <v>0.1096422332823258</v>
       </c>
       <c r="P5" t="n">
-        <v>88.07958151598588</v>
+        <v>0.08535125651662764</v>
       </c>
       <c r="Q5" t="n">
-        <v>39.59235278438562</v>
+        <v>0.07846944159401653</v>
       </c>
       <c r="R5" t="n">
-        <v>15.8743434065319</v>
+        <v>0.07364413530687934</v>
       </c>
       <c r="S5" t="n">
-        <v>3.994941578866926</v>
+        <v>0.06023792794164287</v>
       </c>
       <c r="T5" t="n">
-        <v>-0.8821927141380018</v>
+        <v>0.06428765210460288</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>510.3548</v>
+        <v>509.9661</v>
       </c>
       <c r="B6" t="n">
-        <v>19.34029345382108</v>
+        <v>0.0625762879202942</v>
       </c>
       <c r="C6" t="n">
-        <v>65.40852563305913</v>
+        <v>0.09431384308841133</v>
       </c>
       <c r="D6" t="n">
-        <v>210.1260962776287</v>
+        <v>0.1228560845258758</v>
       </c>
       <c r="E6" t="n">
-        <v>517.5970836755359</v>
+        <v>0.1249201310442888</v>
       </c>
       <c r="F6" t="n">
-        <v>973.0145837902866</v>
+        <v>0.1524011518519721</v>
       </c>
       <c r="G6" t="n">
-        <v>1619.268586383163</v>
+        <v>0.1693905420530027</v>
       </c>
       <c r="H6" t="n">
-        <v>2321.761991333797</v>
+        <v>0.1638816122896158</v>
       </c>
       <c r="I6" t="n">
-        <v>2911.851651567527</v>
+        <v>0.1630439901512064</v>
       </c>
       <c r="J6" t="n">
-        <v>3340.188720518396</v>
+        <v>0.1532308926454252</v>
       </c>
       <c r="K6" t="n">
-        <v>3497.24765980499</v>
+        <v>0.1503023579932283</v>
       </c>
       <c r="L6" t="n">
-        <v>3374.678696080608</v>
+        <v>0.1693476589076549</v>
       </c>
       <c r="M6" t="n">
-        <v>3022.096806529756</v>
+        <v>0.1448610967514569</v>
       </c>
       <c r="N6" t="n">
-        <v>2453.172233755196</v>
+        <v>0.140963567742384</v>
       </c>
       <c r="O6" t="n">
-        <v>1796.35538176122</v>
+        <v>0.1254194803059859</v>
       </c>
       <c r="P6" t="n">
-        <v>1131.069587202701</v>
+        <v>0.1073084059491113</v>
       </c>
       <c r="Q6" t="n">
-        <v>564.5700630996441</v>
+        <v>0.07172305156377333</v>
       </c>
       <c r="R6" t="n">
-        <v>234.4020597550238</v>
+        <v>0.07234826181817637</v>
       </c>
       <c r="S6" t="n">
-        <v>84.54305558946562</v>
+        <v>0.06462195347446588</v>
       </c>
       <c r="T6" t="n">
-        <v>26.77298695930214</v>
+        <v>0.0658774852303811</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>510.44986</v>
+        <v>510.0628</v>
       </c>
       <c r="B7" t="n">
-        <v>60.36428532006443</v>
+        <v>0.05815100173634149</v>
       </c>
       <c r="C7" t="n">
-        <v>180.6219922152627</v>
+        <v>0.1020730042839276</v>
       </c>
       <c r="D7" t="n">
-        <v>419.7478956875473</v>
+        <v>0.1075692729763307</v>
       </c>
       <c r="E7" t="n">
-        <v>778.2236508906583</v>
+        <v>0.1261791304180656</v>
       </c>
       <c r="F7" t="n">
-        <v>1209.902821255459</v>
+        <v>0.1487648380643902</v>
       </c>
       <c r="G7" t="n">
-        <v>1663.509158008976</v>
+        <v>0.1601624223518827</v>
       </c>
       <c r="H7" t="n">
-        <v>2059.026342931035</v>
+        <v>0.1850894322006621</v>
       </c>
       <c r="I7" t="n">
-        <v>2368.853653712653</v>
+        <v>0.2091883838035779</v>
       </c>
       <c r="J7" t="n">
-        <v>2552.352647338262</v>
+        <v>0.1977006390037211</v>
       </c>
       <c r="K7" t="n">
-        <v>2613.668159319167</v>
+        <v>0.2008798256324346</v>
       </c>
       <c r="L7" t="n">
-        <v>2581.722041703723</v>
+        <v>0.181916085422509</v>
       </c>
       <c r="M7" t="n">
-        <v>2436.019349531269</v>
+        <v>0.1556336837929077</v>
       </c>
       <c r="N7" t="n">
-        <v>2156.981887841298</v>
+        <v>0.1390117582138305</v>
       </c>
       <c r="O7" t="n">
-        <v>1738.496684819503</v>
+        <v>0.1290045262337565</v>
       </c>
       <c r="P7" t="n">
-        <v>1237.103093532692</v>
+        <v>0.09755124004980587</v>
       </c>
       <c r="Q7" t="n">
-        <v>727.573050068999</v>
+        <v>0.07198862171143386</v>
       </c>
       <c r="R7" t="n">
-        <v>357.9046186944083</v>
+        <v>0.07718036863191022</v>
       </c>
       <c r="S7" t="n">
-        <v>149.9116167692091</v>
+        <v>0.07964400654687176</v>
       </c>
       <c r="T7" t="n">
-        <v>56.67915322524536</v>
+        <v>0.05681638094288844</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>510.5449</v>
+        <v>510.1595</v>
       </c>
       <c r="B8" t="n">
-        <v>22.63251213098432</v>
+        <v>0.07974796671054375</v>
       </c>
       <c r="C8" t="n">
-        <v>34.68523017722099</v>
+        <v>0.1268683017754753</v>
       </c>
       <c r="D8" t="n">
-        <v>48.65498071980631</v>
+        <v>0.1843671965628753</v>
       </c>
       <c r="E8" t="n">
-        <v>66.72590583098379</v>
+        <v>0.2149617216295871</v>
       </c>
       <c r="F8" t="n">
-        <v>95.45574751325894</v>
+        <v>0.2436180614196579</v>
       </c>
       <c r="G8" t="n">
-        <v>135.5502766741402</v>
+        <v>0.2520456882903208</v>
       </c>
       <c r="H8" t="n">
-        <v>172.4308876642464</v>
+        <v>0.2356841353210996</v>
       </c>
       <c r="I8" t="n">
-        <v>203.2174667647239</v>
+        <v>0.2272590470521089</v>
       </c>
       <c r="J8" t="n">
-        <v>233.0592072214374</v>
+        <v>0.2471894291549361</v>
       </c>
       <c r="K8" t="n">
-        <v>246.5722535267253</v>
+        <v>0.2307166886532472</v>
       </c>
       <c r="L8" t="n">
-        <v>247.4564700041223</v>
+        <v>0.2277244398718918</v>
       </c>
       <c r="M8" t="n">
-        <v>246.6309502743277</v>
+        <v>0.216314262458621</v>
       </c>
       <c r="N8" t="n">
-        <v>231.4887694588047</v>
+        <v>0.179655116911568</v>
       </c>
       <c r="O8" t="n">
-        <v>194.4383701520708</v>
+        <v>0.138486583376613</v>
       </c>
       <c r="P8" t="n">
-        <v>147.3593212601873</v>
+        <v>0.1301638707133864</v>
       </c>
       <c r="Q8" t="n">
-        <v>94.37541032546117</v>
+        <v>0.1117510248638948</v>
       </c>
       <c r="R8" t="n">
-        <v>52.9757141519848</v>
+        <v>0.08858598390321337</v>
       </c>
       <c r="S8" t="n">
-        <v>28.57915168606156</v>
+        <v>0.04258555618572892</v>
       </c>
       <c r="T8" t="n">
-        <v>17.3854801058882</v>
+        <v>0.04016273304393935</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>510.63994</v>
+        <v>510.2562</v>
       </c>
       <c r="B9" t="n">
-        <v>-1.432948096917785</v>
+        <v>0.2006609586834933</v>
       </c>
       <c r="C9" t="n">
-        <v>-0.352386622975835</v>
+        <v>0.3184261387297395</v>
       </c>
       <c r="D9" t="n">
-        <v>6.903785093319616</v>
+        <v>0.4517940871659508</v>
       </c>
       <c r="E9" t="n">
-        <v>15.02745980657182</v>
+        <v>0.5682290038142251</v>
       </c>
       <c r="F9" t="n">
-        <v>27.43371683362022</v>
+        <v>0.618686393175545</v>
       </c>
       <c r="G9" t="n">
-        <v>41.73895606183338</v>
+        <v>0.6103949615868605</v>
       </c>
       <c r="H9" t="n">
-        <v>54.89769994672843</v>
+        <v>0.623374822857096</v>
       </c>
       <c r="I9" t="n">
-        <v>65.10742916942918</v>
+        <v>0.5831022045187252</v>
       </c>
       <c r="J9" t="n">
-        <v>66.55962605390062</v>
+        <v>0.5447601651947642</v>
       </c>
       <c r="K9" t="n">
-        <v>64.30561258362326</v>
+        <v>0.5249421936381032</v>
       </c>
       <c r="L9" t="n">
-        <v>57.77775014004595</v>
+        <v>0.4895869026934341</v>
       </c>
       <c r="M9" t="n">
-        <v>50.16617138474017</v>
+        <v>0.4534660102828337</v>
       </c>
       <c r="N9" t="n">
-        <v>42.46666756509359</v>
+        <v>0.3233861489058643</v>
       </c>
       <c r="O9" t="n">
-        <v>31.98724146385441</v>
+        <v>0.2571694012666592</v>
       </c>
       <c r="P9" t="n">
-        <v>21.66572222409254</v>
+        <v>0.206886280106727</v>
       </c>
       <c r="Q9" t="n">
-        <v>11.55205669181069</v>
+        <v>0.1625398266998632</v>
       </c>
       <c r="R9" t="n">
-        <v>3.937556300091222</v>
+        <v>0.09963505173455933</v>
       </c>
       <c r="S9" t="n">
-        <v>-0.8829716819075386</v>
+        <v>0.08467875722468678</v>
       </c>
       <c r="T9" t="n">
-        <v>-2.207338571920885</v>
+        <v>0.06826123713929394</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>510.73497</v>
+        <v>510.3528</v>
       </c>
       <c r="B10" t="n">
-        <v>2.233819313726925</v>
+        <v>3.069944777370344</v>
       </c>
       <c r="C10" t="n">
-        <v>5.959410080881767</v>
+        <v>4.219561473040068</v>
       </c>
       <c r="D10" t="n">
-        <v>11.38603011136406</v>
+        <v>5.142471047464476</v>
       </c>
       <c r="E10" t="n">
-        <v>16.9966571709654</v>
+        <v>5.638998902856719</v>
       </c>
       <c r="F10" t="n">
-        <v>21.42180767752004</v>
+        <v>5.609253568375312</v>
       </c>
       <c r="G10" t="n">
-        <v>24.17284281088064</v>
+        <v>5.437380091257374</v>
       </c>
       <c r="H10" t="n">
-        <v>24.38980585218576</v>
+        <v>4.874848721095523</v>
       </c>
       <c r="I10" t="n">
-        <v>23.15974983094353</v>
+        <v>4.099034492566851</v>
       </c>
       <c r="J10" t="n">
-        <v>23.54835592938947</v>
+        <v>3.625660735384891</v>
       </c>
       <c r="K10" t="n">
-        <v>22.53801954048988</v>
+        <v>3.164566918206487</v>
       </c>
       <c r="L10" t="n">
-        <v>21.56173773142232</v>
+        <v>2.827364051841096</v>
       </c>
       <c r="M10" t="n">
-        <v>20.14940085633436</v>
+        <v>2.462336116157082</v>
       </c>
       <c r="N10" t="n">
-        <v>17.335582582008</v>
+        <v>1.925498999487491</v>
       </c>
       <c r="O10" t="n">
-        <v>13.78125545927922</v>
+        <v>1.400831854374561</v>
       </c>
       <c r="P10" t="n">
-        <v>10.22584197521169</v>
+        <v>1.083250664693034</v>
       </c>
       <c r="Q10" t="n">
-        <v>7.16107321443764</v>
+        <v>0.8212309740259122</v>
       </c>
       <c r="R10" t="n">
-        <v>5.388657397969038</v>
+        <v>0.5776863034548577</v>
       </c>
       <c r="S10" t="n">
-        <v>3.410278457346471</v>
+        <v>0.3556519905568138</v>
       </c>
       <c r="T10" t="n">
-        <v>1.557034509135185</v>
+        <v>0.2235125951182896</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>510.83</v>
+        <v>510.4495</v>
       </c>
       <c r="B11" t="n">
-        <v>1.043302085560484</v>
+        <v>56.56162225136027</v>
       </c>
       <c r="C11" t="n">
-        <v>0.8437441677404037</v>
+        <v>81.57663925293107</v>
       </c>
       <c r="D11" t="n">
-        <v>1.257707461101266</v>
+        <v>104.9802020893926</v>
       </c>
       <c r="E11" t="n">
-        <v>1.871430823629118</v>
+        <v>120.9064853713981</v>
       </c>
       <c r="F11" t="n">
-        <v>2.976136126854176</v>
+        <v>122.492233250786</v>
       </c>
       <c r="G11" t="n">
-        <v>4.166626741354388</v>
+        <v>110.664411303902</v>
       </c>
       <c r="H11" t="n">
-        <v>4.790740073611805</v>
+        <v>89.23997372000753</v>
       </c>
       <c r="I11" t="n">
-        <v>5.174901788760287</v>
+        <v>72.07774220312571</v>
       </c>
       <c r="J11" t="n">
-        <v>6.112664617859743</v>
+        <v>58.69494293410695</v>
       </c>
       <c r="K11" t="n">
-        <v>7.124920726213055</v>
+        <v>43.58479855345696</v>
       </c>
       <c r="L11" t="n">
-        <v>7.904140012524808</v>
+        <v>33.53629092492187</v>
       </c>
       <c r="M11" t="n">
-        <v>6.733750759093097</v>
+        <v>25.25397946153875</v>
       </c>
       <c r="N11" t="n">
-        <v>4.992216905473649</v>
+        <v>18.02578201983142</v>
       </c>
       <c r="O11" t="n">
-        <v>3.921881394566745</v>
+        <v>13.57240458243627</v>
       </c>
       <c r="P11" t="n">
-        <v>2.503917691326581</v>
+        <v>10.9786646947083</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.9880690552382431</v>
+        <v>8.273073662600339</v>
       </c>
       <c r="R11" t="n">
-        <v>0.3637657616648869</v>
+        <v>5.487521353246342</v>
       </c>
       <c r="S11" t="n">
-        <v>0.2633656190933647</v>
+        <v>3.486279280690007</v>
       </c>
       <c r="T11" t="n">
-        <v>0.2527958464070017</v>
+        <v>2.398830473787402</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>510.5462</v>
+      </c>
+      <c r="B12" t="n">
+        <v>39.64022764597461</v>
+      </c>
+      <c r="C12" t="n">
+        <v>62.59577197334524</v>
+      </c>
+      <c r="D12" t="n">
+        <v>90.68757636401379</v>
+      </c>
+      <c r="E12" t="n">
+        <v>119.1746353710638</v>
+      </c>
+      <c r="F12" t="n">
+        <v>142.3361869629069</v>
+      </c>
+      <c r="G12" t="n">
+        <v>165.9440995096122</v>
+      </c>
+      <c r="H12" t="n">
+        <v>192.8319647204836</v>
+      </c>
+      <c r="I12" t="n">
+        <v>217.5756884251109</v>
+      </c>
+      <c r="J12" t="n">
+        <v>233.0138728962074</v>
+      </c>
+      <c r="K12" t="n">
+        <v>233.3292117533786</v>
+      </c>
+      <c r="L12" t="n">
+        <v>219.4956061652993</v>
+      </c>
+      <c r="M12" t="n">
+        <v>188.3142125909554</v>
+      </c>
+      <c r="N12" t="n">
+        <v>142.7862234173456</v>
+      </c>
+      <c r="O12" t="n">
+        <v>91.3227059968051</v>
+      </c>
+      <c r="P12" t="n">
+        <v>51.75603511307921</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>28.00239823751436</v>
+      </c>
+      <c r="R12" t="n">
+        <v>16.92953428031896</v>
+      </c>
+      <c r="S12" t="n">
+        <v>11.05392880024112</v>
+      </c>
+      <c r="T12" t="n">
+        <v>7.359519987261502</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>510.6428</v>
+      </c>
+      <c r="B13" t="n">
+        <v>3.058133938800696</v>
+      </c>
+      <c r="C13" t="n">
+        <v>5.558571652289212</v>
+      </c>
+      <c r="D13" t="n">
+        <v>9.814383223532444</v>
+      </c>
+      <c r="E13" t="n">
+        <v>16.07186946198065</v>
+      </c>
+      <c r="F13" t="n">
+        <v>25.0375031521134</v>
+      </c>
+      <c r="G13" t="n">
+        <v>36.656409982157</v>
+      </c>
+      <c r="H13" t="n">
+        <v>49.15793072314166</v>
+      </c>
+      <c r="I13" t="n">
+        <v>58.57007802120178</v>
+      </c>
+      <c r="J13" t="n">
+        <v>68.390091376604</v>
+      </c>
+      <c r="K13" t="n">
+        <v>80.06854654909912</v>
+      </c>
+      <c r="L13" t="n">
+        <v>90.08656126311368</v>
+      </c>
+      <c r="M13" t="n">
+        <v>107.7500270056635</v>
+      </c>
+      <c r="N13" t="n">
+        <v>139.1150750708026</v>
+      </c>
+      <c r="O13" t="n">
+        <v>172.9874334942264</v>
+      </c>
+      <c r="P13" t="n">
+        <v>188.3195234490091</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>160.1901814732703</v>
+      </c>
+      <c r="R13" t="n">
+        <v>118.6444081720601</v>
+      </c>
+      <c r="S13" t="n">
+        <v>78.46619174177671</v>
+      </c>
+      <c r="T13" t="n">
+        <v>43.15337562950754</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>510.7395</v>
+      </c>
+      <c r="B14" t="n">
+        <v>0.1937523967550113</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.3619592097847087</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.5900479154811868</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.8467411512755103</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1.312109784842457</v>
+      </c>
+      <c r="G14" t="n">
+        <v>2.042479702294813</v>
+      </c>
+      <c r="H14" t="n">
+        <v>3.663668539092413</v>
+      </c>
+      <c r="I14" t="n">
+        <v>6.525802312114793</v>
+      </c>
+      <c r="J14" t="n">
+        <v>12.56815160525791</v>
+      </c>
+      <c r="K14" t="n">
+        <v>22.09952568134329</v>
+      </c>
+      <c r="L14" t="n">
+        <v>31.10856739009195</v>
+      </c>
+      <c r="M14" t="n">
+        <v>37.15950023575597</v>
+      </c>
+      <c r="N14" t="n">
+        <v>40.50453888667904</v>
+      </c>
+      <c r="O14" t="n">
+        <v>41.11252780780334</v>
+      </c>
+      <c r="P14" t="n">
+        <v>40.40408003102348</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>35.35144102776464</v>
+      </c>
+      <c r="R14" t="n">
+        <v>32.98515963150793</v>
+      </c>
+      <c r="S14" t="n">
+        <v>32.8608530038545</v>
+      </c>
+      <c r="T14" t="n">
+        <v>33.7457384732371</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>510.8361</v>
+      </c>
+      <c r="B15" t="n">
+        <v>0.1225824834086369</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.1729768138409406</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.2095878847891677</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.2711048121899814</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.3798781056181888</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.4846673104429453</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.5478819854189234</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.6181990149723784</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.7685481329727233</v>
+      </c>
+      <c r="K15" t="n">
+        <v>1.38004863752347</v>
+      </c>
+      <c r="L15" t="n">
+        <v>3.068630239345083</v>
+      </c>
+      <c r="M15" t="n">
+        <v>5.791077777170888</v>
+      </c>
+      <c r="N15" t="n">
+        <v>10.51514259607108</v>
+      </c>
+      <c r="O15" t="n">
+        <v>16.19713293527721</v>
+      </c>
+      <c r="P15" t="n">
+        <v>21.05196072680859</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>20.27338641165477</v>
+      </c>
+      <c r="R15" t="n">
+        <v>18.17611118510449</v>
+      </c>
+      <c r="S15" t="n">
+        <v>15.56389124973375</v>
+      </c>
+      <c r="T15" t="n">
+        <v>13.12873901433098</v>
       </c>
     </row>
   </sheetData>

</xml_diff>